<commit_message>
Updated variables from calibration
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SoCEUtiNTY/Share of Cpnt E Use that is New This Year.xlsx
+++ b/InputData/bldgs/SoCEUtiNTY/Share of Cpnt E Use that is New This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\bldgs\SoCEUtiNTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\EPS Structure Research\eps-us-calibration\InputData\bldgs\SoCEUtiNTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{135EE81B-F606-4154-974A-D0CE50805DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2F26AE-BEF3-4DF6-94D2-FC5A4CABA15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="908" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="10008" tabRatio="908" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="calcs&gt;" sheetId="8" r:id="rId6"/>
     <sheet name="Calculations" sheetId="9" r:id="rId7"/>
     <sheet name="Pre-Calibration Calculated Vals" sheetId="10" r:id="rId8"/>
-    <sheet name="SoCEUtiNTY" sheetId="11" r:id="rId9"/>
+    <sheet name="Calibration" sheetId="14" r:id="rId9"/>
+    <sheet name="SoCEUtiNTY" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="598">
   <si>
     <t>Share of New Components Energy Use (dimensionless)</t>
   </si>
@@ -1802,6 +1803,39 @@
   </si>
   <si>
     <t>Alternative electricity and transportation: Table 4, Table 5</t>
+  </si>
+  <si>
+    <t>Calibrated share of component energy use that is new this year (SoCEUtiNTY)</t>
+  </si>
+  <si>
+    <t>Solved offline by calibration/steps/02-bldgs-turnover/solve.py from the BAU export and confirmed by a headless run: the share for each component and building type is the value at which 'Retiring Components Potential Energy Use' at the handoff year (IT + component lifetime, bldgs/CL) equals the new components' energy use in the start year, so retirements show no step. The pre-calibration values (1 / lifetime with hand adjustments) are kept in the 'Pre-Calibration Calculated Vals' tab and column C here. Envelope stays 0 (uses no energy).</t>
+  </si>
+  <si>
+    <t>Building component</t>
+  </si>
+  <si>
+    <t>Building type</t>
+  </si>
+  <si>
+    <t>Pre-calibration share</t>
+  </si>
+  <si>
+    <t>CALIBRATED SHARE USED IN THE OUTPUT TAB</t>
+  </si>
+  <si>
+    <t>Component lifetime (yr)</t>
+  </si>
+  <si>
+    <t>Handoff year</t>
+  </si>
+  <si>
+    <t>Calibration record (2026-09-22)</t>
+  </si>
+  <si>
+    <t>Output values now reference the Calibration tab (calibration/steps/02-bldgs-turnover/solve.py, confirmed by a headless run,</t>
+  </si>
+  <si>
+    <t>retirement step at every handoff 0.0%). The prior 1/lifetime derivation is preserved in 'Pre-Calibration Calculated Vals'.</t>
   </si>
 </sst>
 </file>
@@ -2026,7 +2060,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2057,6 +2091,9 @@
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="34">
     <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
@@ -2394,18 +2431,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B45"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B49"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -2413,174 +2450,189 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="14">
         <v>2025</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B13" s="14">
         <v>2026</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B21" s="14">
         <v>2020</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B23" s="18" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B27" s="15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -2592,13 +2644,148 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="16">
+        <f>Calibration!$D$5</f>
+        <v>4.6808785210000002E-2</v>
+      </c>
+      <c r="C2" s="4">
+        <f>Calibration!$D$10</f>
+        <v>4.6809852220000003E-2</v>
+      </c>
+      <c r="D2" s="16">
+        <f>Calibration!$D$15</f>
+        <v>4.9091647600000003E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="16">
+        <f>Calibration!$D$6</f>
+        <v>6.5652955260000007E-2</v>
+      </c>
+      <c r="C3" s="4">
+        <f>Calibration!$D$11</f>
+        <v>6.5668905969999997E-2</v>
+      </c>
+      <c r="D3" s="16">
+        <f>Calibration!$D$16</f>
+        <v>5.762900713E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="5">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="16">
+        <f>Calibration!$D$7</f>
+        <v>0.11383760580000001</v>
+      </c>
+      <c r="C5" s="4">
+        <f>Calibration!$D$12</f>
+        <v>0.1138513751</v>
+      </c>
+      <c r="D5" s="16">
+        <f>Calibration!$D$17</f>
+        <v>0.1132816153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="16">
+        <f>Calibration!$D$8</f>
+        <v>7.2467006489999999E-2</v>
+      </c>
+      <c r="C6" s="4">
+        <f>Calibration!$D$13</f>
+        <v>7.2458706279999993E-2</v>
+      </c>
+      <c r="D6" s="16">
+        <f>Calibration!$D$18</f>
+        <v>7.1032754510000004E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="16">
+        <f>Calibration!$D$9</f>
+        <v>6.4990485979999998E-2</v>
+      </c>
+      <c r="C7" s="4">
+        <f>Calibration!$D$14</f>
+        <v>6.5000180360000007E-2</v>
+      </c>
+      <c r="D7" s="16">
+        <f>Calibration!$D$19</f>
+        <v>6.5136636509999998E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2607,13 +2794,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.3984375" customWidth="1"/>
-    <col min="2" max="2" width="14.3984375" customWidth="1"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -2621,7 +2808,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2629,7 +2816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2637,7 +2824,7 @@
         <v>15.83333333333333</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2645,7 +2832,7 @@
         <v>51.81818181818182</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -2653,7 +2840,7 @@
         <v>9.1324200913242013</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2661,7 +2848,7 @@
         <v>13.53333333333333</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2677,32 +2864,32 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:AE125"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>50</v>
       </c>
@@ -2794,17 +2981,17 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -2899,7 +3086,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -2994,7 +3181,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -3089,7 +3276,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -3184,7 +3371,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -3279,17 +3466,17 @@
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>63</v>
       </c>
@@ -3384,7 +3571,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>65</v>
       </c>
@@ -3479,12 +3666,12 @@
         <v>170</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>63</v>
       </c>
@@ -3579,7 +3766,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -3674,17 +3861,17 @@
         <v>176</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>69</v>
       </c>
@@ -3779,7 +3966,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -3874,7 +4061,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -3969,7 +4156,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -4064,7 +4251,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -4159,7 +4346,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -4254,7 +4441,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -4349,7 +4536,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>77</v>
       </c>
@@ -4444,7 +4631,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>78</v>
       </c>
@@ -4539,7 +4726,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>79</v>
       </c>
@@ -4634,7 +4821,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -4729,7 +4916,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>81</v>
       </c>
@@ -4824,7 +5011,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -4919,7 +5106,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>83</v>
       </c>
@@ -5014,7 +5201,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -5109,7 +5296,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>85</v>
       </c>
@@ -5204,7 +5391,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>86</v>
       </c>
@@ -5299,7 +5486,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>87</v>
       </c>
@@ -5394,12 +5581,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>69</v>
       </c>
@@ -5494,7 +5681,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>71</v>
       </c>
@@ -5589,7 +5776,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>72</v>
       </c>
@@ -5684,7 +5871,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="44" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>74</v>
       </c>
@@ -5779,7 +5966,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="45" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -5874,7 +6061,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="46" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>83</v>
       </c>
@@ -5969,7 +6156,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="47" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>89</v>
       </c>
@@ -6064,12 +6251,12 @@
         <v>242</v>
       </c>
     </row>
-    <row r="48" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>69</v>
       </c>
@@ -6164,7 +6351,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="50" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>72</v>
       </c>
@@ -6259,7 +6446,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="51" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>83</v>
       </c>
@@ -6354,7 +6541,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>89</v>
       </c>
@@ -6449,12 +6636,12 @@
         <v>245</v>
       </c>
     </row>
-    <row r="53" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="54" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>69</v>
       </c>
@@ -6549,7 +6736,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="55" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>72</v>
       </c>
@@ -6644,7 +6831,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="56" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>74</v>
       </c>
@@ -6739,7 +6926,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="57" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>83</v>
       </c>
@@ -6834,7 +7021,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="58" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>89</v>
       </c>
@@ -6929,7 +7116,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="59" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>92</v>
       </c>
@@ -7024,12 +7211,12 @@
         <v>245</v>
       </c>
     </row>
-    <row r="60" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -7124,7 +7311,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="62" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>71</v>
       </c>
@@ -7219,7 +7406,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="63" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>72</v>
       </c>
@@ -7314,7 +7501,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="64" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>73</v>
       </c>
@@ -7409,7 +7596,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="65" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>74</v>
       </c>
@@ -7504,7 +7691,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="66" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>75</v>
       </c>
@@ -7599,7 +7786,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="67" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>76</v>
       </c>
@@ -7694,7 +7881,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="68" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>77</v>
       </c>
@@ -7789,7 +7976,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="69" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>78</v>
       </c>
@@ -7884,7 +8071,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="70" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -7979,7 +8166,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="71" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>80</v>
       </c>
@@ -8074,7 +8261,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="72" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>81</v>
       </c>
@@ -8169,7 +8356,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="73" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>82</v>
       </c>
@@ -8264,7 +8451,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="74" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -8359,7 +8546,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="75" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -8454,7 +8641,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="76" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>85</v>
       </c>
@@ -8549,7 +8736,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="77" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -8644,7 +8831,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="78" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>89</v>
       </c>
@@ -8739,7 +8926,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="79" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>45</v>
       </c>
@@ -8834,12 +9021,12 @@
         <v>167</v>
       </c>
     </row>
-    <row r="80" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="81" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>69</v>
       </c>
@@ -8934,7 +9121,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="82" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>71</v>
       </c>
@@ -9029,7 +9216,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="83" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>72</v>
       </c>
@@ -9124,7 +9311,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="84" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>73</v>
       </c>
@@ -9219,7 +9406,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="85" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>74</v>
       </c>
@@ -9314,7 +9501,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="86" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>75</v>
       </c>
@@ -9409,7 +9596,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="87" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>76</v>
       </c>
@@ -9504,7 +9691,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="88" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>77</v>
       </c>
@@ -9599,7 +9786,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="89" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>78</v>
       </c>
@@ -9694,7 +9881,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="90" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>79</v>
       </c>
@@ -9789,7 +9976,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="91" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>80</v>
       </c>
@@ -9884,7 +10071,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="92" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>81</v>
       </c>
@@ -9979,7 +10166,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="93" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>82</v>
       </c>
@@ -10074,7 +10261,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="94" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>83</v>
       </c>
@@ -10169,7 +10356,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="95" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>95</v>
       </c>
@@ -10264,7 +10451,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="96" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>85</v>
       </c>
@@ -10359,7 +10546,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>86</v>
       </c>
@@ -10454,7 +10641,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="98" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>96</v>
       </c>
@@ -10549,12 +10736,12 @@
         <v>196</v>
       </c>
     </row>
-    <row r="99" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="100" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>98</v>
       </c>
@@ -10649,7 +10836,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="101" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>99</v>
       </c>
@@ -10744,7 +10931,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="102" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>100</v>
       </c>
@@ -10839,7 +11026,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="103" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>58</v>
       </c>
@@ -10934,12 +11121,12 @@
         <v>362</v>
       </c>
     </row>
-    <row r="104" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="105" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>101</v>
       </c>
@@ -11034,7 +11221,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="106" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>103</v>
       </c>
@@ -11129,7 +11316,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="107" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>104</v>
       </c>
@@ -11224,7 +11411,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="108" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>105</v>
       </c>
@@ -11319,7 +11506,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="109" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>106</v>
       </c>
@@ -11414,7 +11601,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="110" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>107</v>
       </c>
@@ -11509,7 +11696,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="111" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>108</v>
       </c>
@@ -11604,7 +11791,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="112" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>109</v>
       </c>
@@ -11699,7 +11886,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="113" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>110</v>
       </c>
@@ -11794,7 +11981,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="114" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>111</v>
       </c>
@@ -11889,12 +12076,12 @@
         <v>344</v>
       </c>
     </row>
-    <row r="115" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="116" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>101</v>
       </c>
@@ -11989,7 +12176,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="117" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>103</v>
       </c>
@@ -12084,7 +12271,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="118" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>104</v>
       </c>
@@ -12179,7 +12366,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="119" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>105</v>
       </c>
@@ -12274,7 +12461,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="120" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>106</v>
       </c>
@@ -12369,7 +12556,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="121" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>107</v>
       </c>
@@ -12464,7 +12651,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="122" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>108</v>
       </c>
@@ -12559,7 +12746,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="123" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>109</v>
       </c>
@@ -12654,7 +12841,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="124" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>110</v>
       </c>
@@ -12749,7 +12936,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="125" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>111</v>
       </c>
@@ -12852,29 +13039,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:AE102"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>50</v>
       </c>
@@ -12966,17 +13153,17 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>115</v>
       </c>
@@ -13071,7 +13258,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -13166,7 +13353,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>58</v>
       </c>
@@ -13261,17 +13448,17 @@
         <v>203</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -13366,7 +13553,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -13461,17 +13648,17 @@
         <v>365</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -13566,7 +13753,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -13661,7 +13848,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>72</v>
       </c>
@@ -13756,7 +13943,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>119</v>
       </c>
@@ -13851,7 +14038,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -13946,7 +14133,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -14041,7 +14228,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -14136,7 +14323,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>432</v>
       </c>
@@ -14231,7 +14418,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>436</v>
       </c>
@@ -14326,7 +14513,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>83</v>
       </c>
@@ -14421,7 +14608,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>84</v>
       </c>
@@ -14516,7 +14703,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>85</v>
       </c>
@@ -14611,7 +14798,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -14706,7 +14893,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>120</v>
       </c>
@@ -14801,12 +14988,12 @@
         <v>237</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>69</v>
       </c>
@@ -14901,7 +15088,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>71</v>
       </c>
@@ -14996,7 +15183,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>72</v>
       </c>
@@ -15091,7 +15278,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -15186,7 +15373,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>83</v>
       </c>
@@ -15281,7 +15468,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>89</v>
       </c>
@@ -15376,12 +15563,12 @@
         <v>463</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -15476,7 +15663,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>72</v>
       </c>
@@ -15571,7 +15758,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -15666,7 +15853,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>89</v>
       </c>
@@ -15761,7 +15948,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>121</v>
       </c>
@@ -15856,7 +16043,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="44" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>122</v>
       </c>
@@ -15951,12 +16138,12 @@
         <v>443</v>
       </c>
     </row>
-    <row r="45" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>69</v>
       </c>
@@ -16051,7 +16238,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="47" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>71</v>
       </c>
@@ -16146,7 +16333,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="48" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>72</v>
       </c>
@@ -16241,7 +16428,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="49" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>119</v>
       </c>
@@ -16336,7 +16523,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="50" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>74</v>
       </c>
@@ -16431,7 +16618,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="51" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>77</v>
       </c>
@@ -16526,7 +16713,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>73</v>
       </c>
@@ -16621,7 +16808,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="53" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>432</v>
       </c>
@@ -16716,7 +16903,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="54" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>436</v>
       </c>
@@ -16811,7 +16998,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="55" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>83</v>
       </c>
@@ -16906,7 +17093,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="56" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -17001,7 +17188,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="57" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>85</v>
       </c>
@@ -17096,7 +17283,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="58" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>86</v>
       </c>
@@ -17191,7 +17378,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="59" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>89</v>
       </c>
@@ -17286,7 +17473,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="60" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>45</v>
       </c>
@@ -17381,12 +17568,12 @@
         <v>463</v>
       </c>
     </row>
-    <row r="61" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="62" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>69</v>
       </c>
@@ -17481,7 +17668,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="63" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>71</v>
       </c>
@@ -17576,7 +17763,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="64" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -17671,7 +17858,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="65" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>119</v>
       </c>
@@ -17766,7 +17953,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -17861,7 +18048,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="67" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>77</v>
       </c>
@@ -17956,7 +18143,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="68" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -18051,7 +18238,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="69" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>432</v>
       </c>
@@ -18146,7 +18333,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="70" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>436</v>
       </c>
@@ -18241,7 +18428,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="71" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -18336,7 +18523,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="72" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>95</v>
       </c>
@@ -18431,7 +18618,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="73" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>85</v>
       </c>
@@ -18526,7 +18713,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="74" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>86</v>
       </c>
@@ -18621,7 +18808,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="75" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>96</v>
       </c>
@@ -18716,12 +18903,12 @@
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="77" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>124</v>
       </c>
@@ -18816,7 +19003,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="78" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>99</v>
       </c>
@@ -18911,7 +19098,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="79" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>100</v>
       </c>
@@ -19006,7 +19193,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="80" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>58</v>
       </c>
@@ -19101,12 +19288,12 @@
         <v>544</v>
       </c>
     </row>
-    <row r="81" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="82" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>101</v>
       </c>
@@ -19201,7 +19388,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="83" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>103</v>
       </c>
@@ -19296,7 +19483,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="84" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>104</v>
       </c>
@@ -19391,7 +19578,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="85" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>105</v>
       </c>
@@ -19486,7 +19673,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="86" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>106</v>
       </c>
@@ -19581,7 +19768,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>107</v>
       </c>
@@ -19676,7 +19863,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="88" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>108</v>
       </c>
@@ -19771,7 +19958,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="89" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>109</v>
       </c>
@@ -19866,7 +20053,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="90" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>110</v>
       </c>
@@ -19961,7 +20148,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="91" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>111</v>
       </c>
@@ -20056,12 +20243,12 @@
         <v>344</v>
       </c>
     </row>
-    <row r="92" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="93" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>101</v>
       </c>
@@ -20156,7 +20343,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="94" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>103</v>
       </c>
@@ -20251,7 +20438,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="95" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>104</v>
       </c>
@@ -20346,7 +20533,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="96" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>105</v>
       </c>
@@ -20441,7 +20628,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="97" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>106</v>
       </c>
@@ -20536,7 +20723,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="98" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>107</v>
       </c>
@@ -20631,7 +20818,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="99" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>108</v>
       </c>
@@ -20726,7 +20913,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="100" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>109</v>
       </c>
@@ -20821,7 +21008,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="101" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>110</v>
       </c>
@@ -20916,7 +21103,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="102" spans="1:31" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>111</v>
       </c>
@@ -21022,7 +21209,7 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21031,21 +21218,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:AC67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="13.1328125" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>125</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B2">
         <v>2025</v>
       </c>
@@ -21125,7 +21312,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>126</v>
       </c>
@@ -21235,7 +21422,7 @@
       </c>
       <c r="AB3" s="6"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -21244,19 +21431,19 @@
         <v>2.4515798493830544E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>127</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
         <v>129</v>
       </c>
@@ -21264,7 +21451,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>131</v>
       </c>
@@ -21272,7 +21459,7 @@
         <v>0.997</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>132</v>
       </c>
@@ -21280,7 +21467,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -21288,12 +21475,12 @@
         <v>0.96599999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>2025</v>
       </c>
@@ -21373,7 +21560,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>131</v>
       </c>
@@ -21484,7 +21671,7 @@
       <c r="AB19" s="11"/>
       <c r="AC19" s="11"/>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>132</v>
       </c>
@@ -21595,7 +21782,7 @@
       <c r="AB20" s="11"/>
       <c r="AC20" s="11"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>133</v>
       </c>
@@ -21706,13 +21893,13 @@
       <c r="AB21" s="11"/>
       <c r="AC21" s="11"/>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>135</v>
       </c>
       <c r="D23" s="11"/>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>2025</v>
       </c>
@@ -21792,7 +21979,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>131</v>
       </c>
@@ -21903,7 +22090,7 @@
       <c r="AB25" s="11"/>
       <c r="AC25" s="11"/>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>132</v>
       </c>
@@ -22014,7 +22201,7 @@
       <c r="AB26" s="11"/>
       <c r="AC26" s="11"/>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>133</v>
       </c>
@@ -22125,12 +22312,12 @@
       <c r="AB27" s="11"/>
       <c r="AC27" s="11"/>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>2025</v>
       </c>
@@ -22210,348 +22397,348 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>131</v>
       </c>
       <c r="B31" s="6">
-        <f>B25/B19</f>
+        <f t="shared" ref="B31:AA31" si="0">B25/B19</f>
         <v>3.0090270812437548E-3</v>
       </c>
       <c r="C31" s="6">
-        <f>C25/C19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437861E-3</v>
       </c>
       <c r="D31" s="6">
-        <f>D25/D19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437583E-3</v>
       </c>
       <c r="E31" s="6">
-        <f>E25/E19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437444E-3</v>
       </c>
       <c r="F31" s="6">
-        <f>F25/F19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437787E-3</v>
       </c>
       <c r="G31" s="6">
-        <f>G25/G19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437813E-3</v>
       </c>
       <c r="H31" s="6">
-        <f>H25/H19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437583E-3</v>
       </c>
       <c r="I31" s="6">
-        <f>I25/I19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437292E-3</v>
       </c>
       <c r="J31" s="6">
-        <f>J25/J19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437787E-3</v>
       </c>
       <c r="K31" s="6">
-        <f>K25/K19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437349E-3</v>
       </c>
       <c r="L31" s="6">
-        <f>L25/L19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437089E-3</v>
       </c>
       <c r="M31" s="6">
-        <f>M25/M19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812436711E-3</v>
       </c>
       <c r="N31" s="6">
-        <f>N25/N19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437704E-3</v>
       </c>
       <c r="O31" s="6">
-        <f>O25/O19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437054E-3</v>
       </c>
       <c r="P31" s="6">
-        <f>P25/P19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437162E-3</v>
       </c>
       <c r="Q31" s="6">
-        <f>Q25/Q19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437145E-3</v>
       </c>
       <c r="R31" s="6">
-        <f>R25/R19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437449E-3</v>
       </c>
       <c r="S31" s="6">
-        <f>S25/S19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437388E-3</v>
       </c>
       <c r="T31" s="6">
-        <f>T25/T19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812436824E-3</v>
       </c>
       <c r="U31" s="6">
-        <f>U25/U19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437752E-3</v>
       </c>
       <c r="V31" s="6">
-        <f>V25/V19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812436902E-3</v>
       </c>
       <c r="W31" s="6">
-        <f>W25/W19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437427E-3</v>
       </c>
       <c r="X31" s="6">
-        <f>X25/X19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812436729E-3</v>
       </c>
       <c r="Y31" s="6">
-        <f>Y25/Y19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437787E-3</v>
       </c>
       <c r="Z31" s="6">
-        <f>Z25/Z19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437921E-3</v>
       </c>
       <c r="AA31" s="6">
-        <f>AA25/AA19</f>
+        <f t="shared" si="0"/>
         <v>3.0090270812437687E-3</v>
       </c>
       <c r="AB31" s="6"/>
       <c r="AC31" s="6"/>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>132</v>
       </c>
       <c r="B32" s="6">
-        <f>B26/B20</f>
+        <f t="shared" ref="B32:AA32" si="1">B26/B20</f>
         <v>5.0251256281406819E-3</v>
       </c>
       <c r="C32" s="6">
-        <f>C26/C20</f>
+        <f t="shared" si="1"/>
         <v>5.025125628140675E-3</v>
       </c>
       <c r="D32" s="6">
-        <f>D26/D20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406559E-3</v>
       </c>
       <c r="E32" s="6">
-        <f>E26/E20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407799E-3</v>
       </c>
       <c r="F32" s="6">
-        <f>F26/F20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406307E-3</v>
       </c>
       <c r="G32" s="6">
-        <f>G26/G20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407565E-3</v>
       </c>
       <c r="H32" s="6">
-        <f>H26/H20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406871E-3</v>
       </c>
       <c r="I32" s="6">
-        <f>I26/I20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406247E-3</v>
       </c>
       <c r="J32" s="6">
-        <f>J26/J20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406273E-3</v>
       </c>
       <c r="K32" s="6">
-        <f>K26/K20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406568E-3</v>
       </c>
       <c r="L32" s="6">
-        <f>L26/L20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406576E-3</v>
       </c>
       <c r="M32" s="6">
-        <f>M26/M20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407886E-3</v>
       </c>
       <c r="N32" s="6">
-        <f>N26/N20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406767E-3</v>
       </c>
       <c r="O32" s="6">
-        <f>O26/O20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407704E-3</v>
       </c>
       <c r="P32" s="6">
-        <f>P26/P20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406706E-3</v>
       </c>
       <c r="Q32" s="6">
-        <f>Q26/Q20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407166E-3</v>
       </c>
       <c r="R32" s="6">
-        <f>R26/R20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407608E-3</v>
       </c>
       <c r="S32" s="6">
-        <f>S26/S20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406715E-3</v>
       </c>
       <c r="T32" s="6">
-        <f>T26/T20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406533E-3</v>
       </c>
       <c r="U32" s="6">
-        <f>U26/U20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407834E-3</v>
       </c>
       <c r="V32" s="6">
-        <f>V26/V20</f>
+        <f t="shared" si="1"/>
         <v>5.025125628140629E-3</v>
       </c>
       <c r="W32" s="6">
-        <f>W26/W20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406568E-3</v>
       </c>
       <c r="X32" s="6">
-        <f>X26/X20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406914E-3</v>
       </c>
       <c r="Y32" s="6">
-        <f>Y26/Y20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281407643E-3</v>
       </c>
       <c r="Z32" s="6">
-        <f>Z26/Z20</f>
+        <f t="shared" si="1"/>
         <v>5.025125628140773E-3</v>
       </c>
       <c r="AA32" s="6">
-        <f>AA26/AA20</f>
+        <f t="shared" si="1"/>
         <v>5.0251256281406802E-3</v>
       </c>
       <c r="AB32" s="6"/>
       <c r="AC32" s="6"/>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>133</v>
       </c>
       <c r="B33" s="6">
-        <f>B27/B21</f>
+        <f t="shared" ref="B33:AA33" si="2">B27/B21</f>
         <v>3.5196687370600402E-2</v>
       </c>
       <c r="C33" s="6">
-        <f>C27/C21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600374E-2</v>
       </c>
       <c r="D33" s="6">
-        <f>D27/D21</f>
+        <f t="shared" si="2"/>
         <v>3.519668737060045E-2</v>
       </c>
       <c r="E33" s="6">
-        <f>E27/E21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600457E-2</v>
       </c>
       <c r="F33" s="6">
-        <f>F27/F21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600471E-2</v>
       </c>
       <c r="G33" s="6">
-        <f>G27/G21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600457E-2</v>
       </c>
       <c r="H33" s="6">
-        <f>H27/H21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600492E-2</v>
       </c>
       <c r="I33" s="6">
-        <f>I27/I21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600402E-2</v>
       </c>
       <c r="J33" s="6">
-        <f>J27/J21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600457E-2</v>
       </c>
       <c r="K33" s="6">
-        <f>K27/K21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600492E-2</v>
       </c>
       <c r="L33" s="6">
-        <f>L27/L21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600444E-2</v>
       </c>
       <c r="M33" s="6">
-        <f>M27/M21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600395E-2</v>
       </c>
       <c r="N33" s="6">
-        <f>N27/N21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600388E-2</v>
       </c>
       <c r="O33" s="6">
-        <f>O27/O21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600457E-2</v>
       </c>
       <c r="P33" s="6">
-        <f>P27/P21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600437E-2</v>
       </c>
       <c r="Q33" s="6">
-        <f>Q27/Q21</f>
+        <f t="shared" si="2"/>
         <v>3.519668737060043E-2</v>
       </c>
       <c r="R33" s="6">
-        <f>R27/R21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600471E-2</v>
       </c>
       <c r="S33" s="6">
-        <f>S27/S21</f>
+        <f t="shared" si="2"/>
         <v>3.519668737060045E-2</v>
       </c>
       <c r="T33" s="6">
-        <f>T27/T21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600416E-2</v>
       </c>
       <c r="U33" s="6">
-        <f>U27/U21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600492E-2</v>
       </c>
       <c r="V33" s="6">
-        <f>V27/V21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600506E-2</v>
       </c>
       <c r="W33" s="6">
-        <f>W27/W21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600409E-2</v>
       </c>
       <c r="X33" s="6">
-        <f>X27/X21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600457E-2</v>
       </c>
       <c r="Y33" s="6">
-        <f>Y27/Y21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600478E-2</v>
       </c>
       <c r="Z33" s="6">
-        <f>Z27/Z21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600423E-2</v>
       </c>
       <c r="AA33" s="6">
-        <f>AA27/AA21</f>
+        <f t="shared" si="2"/>
         <v>3.5196687370600506E-2</v>
       </c>
       <c r="AB33" s="6"/>
       <c r="AC33" s="6"/>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
       <c r="C34" s="7"/>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>131</v>
       </c>
@@ -22560,30 +22747,30 @@
         <v>3.0090270812437414E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>132</v>
       </c>
       <c r="B37" s="8">
-        <f t="shared" ref="B37:B38" si="0">AVERAGE(B32:AA32)</f>
+        <f t="shared" ref="B37:B38" si="3">AVERAGE(B32:AA32)</f>
         <v>5.0251256281406967E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>133</v>
       </c>
       <c r="B38" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.519668737060045E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>139</v>
       </c>
@@ -22592,34 +22779,34 @@
         <v>5.2007924082897363E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
         <v>140</v>
       </c>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
     </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>145</v>
       </c>
@@ -22628,7 +22815,7 @@
         <v>0.97548420150616943</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>146</v>
       </c>
@@ -22637,12 +22824,12 @@
         <v>0.99479920759171026</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -22651,7 +22838,7 @@
         <v>5.2631578947368418E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>5</v>
       </c>
@@ -22660,7 +22847,7 @@
         <v>6.3157894736842121E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>7</v>
       </c>
@@ -22669,7 +22856,7 @@
         <v>0.1095</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -22678,7 +22865,7 @@
         <v>7.3891625615763568E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>9</v>
       </c>
@@ -22687,12 +22874,12 @@
         <v>6.4935064935064929E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>145</v>
       </c>
@@ -22700,7 +22887,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>4</v>
       </c>
@@ -22713,7 +22900,7 @@
         <v>5.7558645439432378E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>5</v>
       </c>
@@ -22726,7 +22913,7 @@
         <v>6.8030216045660924E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>7</v>
       </c>
@@ -22739,7 +22926,7 @@
         <v>0.114131305639582</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -22752,7 +22939,7 @@
         <v>7.8708123018514653E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>9</v>
       </c>
@@ -22774,15 +22961,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.73046875" customWidth="1"/>
-    <col min="2" max="2" width="17.53125" customWidth="1"/>
-    <col min="3" max="3" width="18.265625" customWidth="1"/>
-    <col min="4" max="4" width="14.86328125" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
@@ -22793,7 +22980,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -22810,7 +22997,7 @@
         <v>7.5857072257313141E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -22827,7 +23014,7 @@
         <v>8.6125327010009689E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -22841,7 +23028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -22858,7 +23045,7 @@
         <v>0.1313313185587561</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -22875,7 +23062,7 @@
         <v>9.6595911905616477E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -22892,7 +23079,7 @@
         <v>8.785892846176363E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D8" s="4"/>
     </row>
   </sheetData>
@@ -22901,132 +23088,354 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03FEDAA-BDD5-4838-BC55-9E4145665C32}">
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.73046875" customWidth="1"/>
-    <col min="2" max="2" width="17.53125" customWidth="1"/>
-    <col min="3" max="3" width="18.265625" customWidth="1"/>
-    <col min="4" max="4" width="14.86328125" customWidth="1"/>
+    <col min="1" max="8" width="20.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>588</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+    </row>
+    <row r="4" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>589</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>590</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>591</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>592</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C5">
+        <v>5.2631578950000001E-2</v>
+      </c>
+      <c r="D5">
+        <v>4.6808785210000002E-2</v>
+      </c>
+      <c r="E5">
+        <v>19</v>
+      </c>
+      <c r="F5">
+        <v>2044</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>6.3157894739999998E-2</v>
+      </c>
+      <c r="D6">
+        <v>6.5652955260000007E-2</v>
+      </c>
+      <c r="E6">
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0.1095</v>
+      </c>
+      <c r="D7">
+        <v>0.11383760580000001</v>
+      </c>
+      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="F7">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="D8">
+        <v>7.2467006489999999E-2</v>
+      </c>
+      <c r="E8">
+        <v>14</v>
+      </c>
+      <c r="F8">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="D9">
+        <v>6.4990485979999998E-2</v>
+      </c>
+      <c r="E9">
+        <v>15</v>
+      </c>
+      <c r="F9">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="C10">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="D10">
+        <v>4.6809852220000003E-2</v>
+      </c>
+      <c r="E10">
+        <v>19</v>
+      </c>
+      <c r="F10">
+        <v>2044</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>6.3157894739999998E-2</v>
+      </c>
+      <c r="D11">
+        <v>6.5668905969999997E-2</v>
+      </c>
+      <c r="E11">
+        <v>16</v>
+      </c>
+      <c r="F11">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12">
+        <v>0.1095</v>
+      </c>
+      <c r="D12">
+        <v>0.1138513751</v>
+      </c>
+      <c r="E12">
+        <v>9</v>
+      </c>
+      <c r="F12">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="D13">
+        <v>7.2458706279999993E-2</v>
+      </c>
+      <c r="E13">
+        <v>14</v>
+      </c>
+      <c r="F13">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="D14">
+        <v>6.5000180360000007E-2</v>
+      </c>
+      <c r="E14">
+        <v>15</v>
+      </c>
+      <c r="F14">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="16">
-        <f>1/'Component Lifetimes'!B2</f>
-        <v>5.2631578947368418E-2</v>
-      </c>
-      <c r="C2" s="4">
-        <v>5.2999999999999999E-2</v>
-      </c>
-      <c r="D2" s="16">
-        <f>1/'Component Lifetimes'!B2</f>
-        <v>5.2631578947368418E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="C15">
+        <v>5.2631578950000001E-2</v>
+      </c>
+      <c r="D15">
+        <v>4.9091647600000003E-2</v>
+      </c>
+      <c r="E15">
+        <v>19</v>
+      </c>
+      <c r="F15">
+        <v>2044</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="16">
-        <f>1/'Component Lifetimes'!B3</f>
-        <v>6.3157894736842121E-2</v>
-      </c>
-      <c r="C3" s="4">
-        <f>B3</f>
-        <v>6.3157894736842121E-2</v>
-      </c>
-      <c r="D3" s="16">
-        <f>1/'Component Lifetimes'!B3</f>
-        <v>6.3157894736842121E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="5">
-        <v>0</v>
-      </c>
-      <c r="C4" s="5">
-        <v>0</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>6.3157894739999998E-2</v>
+      </c>
+      <c r="D16">
+        <v>5.762900713E-2</v>
+      </c>
+      <c r="E16">
+        <v>16</v>
+      </c>
+      <c r="F16">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16">
-        <f>1/'Component Lifetimes'!B5</f>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17">
         <v>0.1095</v>
       </c>
-      <c r="C5" s="4">
-        <f>B5</f>
-        <v>0.1095</v>
-      </c>
-      <c r="D5" s="16">
-        <f>1/'Component Lifetimes'!B5</f>
-        <v>0.1095</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="D17">
+        <v>0.1132816153</v>
+      </c>
+      <c r="E17">
+        <v>9</v>
+      </c>
+      <c r="F17">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="C6" s="4">
-        <f>B6</f>
-        <v>7.0999999999999994E-2</v>
-      </c>
-      <c r="D6" s="16">
-        <f>B6</f>
-        <v>7.0999999999999994E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+      <c r="D18">
+        <v>7.1032754510000004E-2</v>
+      </c>
+      <c r="E18">
+        <v>14</v>
+      </c>
+      <c r="F18">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="C7" s="4">
-        <f>B7</f>
-        <v>6.6000000000000003E-2</v>
-      </c>
-      <c r="D7" s="16">
-        <v>6.6000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="D8" s="4"/>
+      <c r="D19">
+        <v>6.5136636509999998E-2</v>
+      </c>
+      <c r="E19">
+        <v>15</v>
+      </c>
+      <c r="F19">
+        <v>2040</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>